<commit_message>
Align trial workbook styling with exact original sheet: Row 1 Cyan header, Row 2 counter, frozen panes, and data starting at Row 3
</commit_message>
<xml_diff>
--- a/UPPCL_X_Complaint_Trial_Workbook.xlsx
+++ b/UPPCL_X_Complaint_Trial_Workbook.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,28 +29,36 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Verdana"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="001A2F40"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Verdana"/>
+      <b val="1"/>
+      <color rgb="001A2F40"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
+      <name val="Verdana"/>
+      <color rgb="001A2F40"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Times New Roman"/>
+      <color rgb="001D9BF0"/>
+      <sz val="11"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Verdana"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="001A2F40"/>
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -59,20 +67,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001A73E8"/>
-        <bgColor rgb="001A73E8"/>
+        <fgColor rgb="004DD0E1"/>
+        <bgColor rgb="004DD0E1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000D652D"/>
-        <bgColor rgb="000D652D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F1F3F4"/>
-        <bgColor rgb="00F1F3F4"/>
+        <fgColor rgb="0000ACC1"/>
+        <bgColor rgb="0000ACC1"/>
       </patternFill>
     </fill>
   </fills>
@@ -86,40 +88,48 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00E0E0E0"/>
+        <color rgb="00000000"/>
       </left>
       <right style="thin">
-        <color rgb="00E0E0E0"/>
+        <color rgb="00000000"/>
       </right>
       <top style="thin">
-        <color rgb="00E0E0E0"/>
+        <color rgb="00000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="00E0E0E0"/>
+        <color rgb="00000000"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -485,1095 +495,1126 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF17"/>
+  <dimension ref="A1:AF9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="21" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="42" customWidth="1" min="14" max="14"/>
-    <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="39" customWidth="1" min="16" max="16"/>
-    <col width="32" customWidth="1" min="17" max="17"/>
-    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="22" customWidth="1" min="20" max="20"/>
-    <col width="50" customWidth="1" min="21" max="21"/>
+    <col width="25" customWidth="1" min="20" max="20"/>
+    <col width="45" customWidth="1" min="21" max="21"/>
     <col width="24" customWidth="1" min="22" max="22"/>
-    <col width="26" customWidth="1" min="23" max="23"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
     <col width="12" customWidth="1" min="24" max="24"/>
-    <col width="21" customWidth="1" min="25" max="25"/>
-    <col width="50" customWidth="1" min="26" max="26"/>
-    <col width="24" customWidth="1" min="27" max="27"/>
-    <col width="16" customWidth="1" min="28" max="28"/>
-    <col width="17" customWidth="1" min="29" max="29"/>
-    <col width="18" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="25" max="25"/>
+    <col width="45" customWidth="1" min="26" max="26"/>
+    <col width="22" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="35" customWidth="1" min="29" max="29"/>
+    <col width="24" customWidth="1" min="30" max="30"/>
     <col width="20" customWidth="1" min="31" max="31"/>
-    <col width="13" customWidth="1" min="32" max="32"/>
+    <col width="25" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+    <row r="1" ht="66" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>DATE</t>
         </is>
       </c>
-      <c r="B9" s="1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Link Shift</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Reply Shift</t>
         </is>
       </c>
-      <c r="D9" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>C F</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve"> LINK URL</t>
         </is>
       </c>
-      <c r="F9" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Twitter Id</t>
         </is>
       </c>
-      <c r="G9" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Head</t>
         </is>
       </c>
-      <c r="H9" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Untagged Complaint</t>
         </is>
       </c>
-      <c r="I9" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Picked Status</t>
         </is>
       </c>
-      <c r="J9" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Complaint Type</t>
         </is>
       </c>
-      <c r="K9" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>DISCOM</t>
         </is>
       </c>
-      <c r="L9" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Zone</t>
         </is>
       </c>
-      <c r="M9" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>District</t>
         </is>
       </c>
-      <c r="N9" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Remark</t>
         </is>
       </c>
-      <c r="O9" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="P9" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>REPLY_WITHIN_30_MIN_BY_Laqshya Media</t>
         </is>
       </c>
-      <c r="Q9" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>REPLY_WITHIN_60_MIN_BY_DISCOM</t>
         </is>
       </c>
-      <c r="R9" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>COMPLAINT_NO</t>
         </is>
       </c>
-      <c r="S9" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>STS</t>
         </is>
       </c>
-      <c r="T9" s="2" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>Post ID</t>
         </is>
       </c>
-      <c r="U9" s="2" t="inlineStr">
+      <c r="U1" s="2" t="inlineStr">
         <is>
           <t>Post Text</t>
         </is>
       </c>
-      <c r="V9" s="2" t="inlineStr">
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>Post Created At (UTC)</t>
         </is>
       </c>
-      <c r="W9" s="2" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>First Detected At (IST)</t>
         </is>
       </c>
-      <c r="X9" s="2" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>Language</t>
         </is>
       </c>
-      <c r="Y9" s="2" t="inlineStr">
+      <c r="Y1" s="2" t="inlineStr">
         <is>
           <t>Routing Confidence</t>
         </is>
       </c>
-      <c r="Z9" s="2" t="inlineStr">
+      <c r="Z1" s="2" t="inlineStr">
         <is>
           <t>Suggested Reply Draft</t>
         </is>
       </c>
-      <c r="AA9" s="2" t="inlineStr">
+      <c r="AA1" s="2" t="inlineStr">
         <is>
           <t>Reply Approval Status</t>
         </is>
       </c>
-      <c r="AB9" s="2" t="inlineStr">
+      <c r="AB1" s="2" t="inlineStr">
         <is>
           <t>Reply Post ID</t>
         </is>
       </c>
-      <c r="AC9" s="2" t="inlineStr">
+      <c r="AC1" s="2" t="inlineStr">
         <is>
           <t>Reply Post URL</t>
         </is>
       </c>
-      <c r="AD9" s="2" t="inlineStr">
+      <c r="AD1" s="2" t="inlineStr">
         <is>
           <t>Reply Posted At</t>
         </is>
       </c>
-      <c r="AE9" s="2" t="inlineStr">
+      <c r="AE1" s="2" t="inlineStr">
         <is>
           <t>Processing Status</t>
         </is>
       </c>
-      <c r="AF9" s="2" t="inlineStr">
+      <c r="AF1" s="2" t="inlineStr">
         <is>
           <t>Last Error</t>
         </is>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="2" ht="33" customHeight="1">
+      <c r="A2" s="3" t="n"/>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
+      <c r="I2" s="3" t="n"/>
+      <c r="J2" s="3">
+        <f>COUNTA(E3:E50)</f>
+        <v/>
+      </c>
+      <c r="K2" s="3" t="n"/>
+      <c r="L2" s="3" t="n"/>
+      <c r="M2" s="3" t="n"/>
+      <c r="N2" s="3" t="n"/>
+      <c r="O2" s="3" t="n"/>
+      <c r="P2" s="3" t="n"/>
+      <c r="Q2" s="3">
+        <f>COUNTIF(Q3:Q50, "YES")</f>
+        <v/>
+      </c>
+      <c r="R2" s="3" t="n"/>
+      <c r="S2" s="3" t="n"/>
+      <c r="T2" s="3" t="n"/>
+      <c r="U2" s="3" t="n"/>
+      <c r="V2" s="3" t="n"/>
+      <c r="W2" s="3" t="n"/>
+      <c r="X2" s="3" t="n"/>
+      <c r="Y2" s="3" t="n"/>
+      <c r="Z2" s="3" t="n"/>
+      <c r="AA2" s="3" t="n"/>
+      <c r="AB2" s="3" t="n"/>
+      <c r="AC2" s="3" t="n"/>
+      <c r="AD2" s="3" t="n"/>
+      <c r="AE2" s="3" t="n"/>
+      <c r="AF2" s="3" t="n"/>
+    </row>
+    <row r="3" ht="45" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>19-10-2026</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>MORNING</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>MORNING</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>https://x.com/Diwaker70180261/status/2111604765486707028?s=20</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Diwaker70180261</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>upm</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr"/>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>SUPPLY_OUTAGE</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>MVVNL</t>
         </is>
       </c>
-      <c r="L11" s="3" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>DEVIPATAN</t>
         </is>
       </c>
-      <c r="M11" s="3" t="inlineStr">
+      <c r="M3" s="4" t="inlineStr">
         <is>
           <t>GONDA</t>
         </is>
       </c>
-      <c r="N11" s="3" t="inlineStr">
+      <c r="N3" s="6" t="inlineStr">
         <is>
           <t>Verified match for GONDA -&gt; MVVNL</t>
         </is>
       </c>
-      <c r="O11" s="3" t="inlineStr">
+      <c r="O3" s="4" t="inlineStr">
         <is>
           <t>Forwarded to Discom</t>
         </is>
       </c>
-      <c r="P11" s="3" t="inlineStr">
+      <c r="P3" s="4" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="Q11" s="3" t="inlineStr"/>
-      <c r="R11" s="3" t="inlineStr"/>
-      <c r="S11" s="3" t="inlineStr"/>
-      <c r="T11" s="3" t="inlineStr">
+      <c r="Q3" s="4" t="inlineStr"/>
+      <c r="R3" s="4" t="inlineStr"/>
+      <c r="S3" s="4" t="inlineStr"/>
+      <c r="T3" s="6" t="inlineStr">
         <is>
           <t>2111604765486707028</t>
         </is>
       </c>
-      <c r="U11" s="3" t="inlineStr">
+      <c r="U3" s="6" t="inlineStr">
         <is>
           <t>@UPPCLLKO @mduppcl गोंडा जिले के वजीरगंज ब्लॉक में पिछले 12 घंटे से बिजली आपूर्ति पूरी तरह बाधित है।</t>
         </is>
       </c>
-      <c r="V11" s="3" t="inlineStr">
+      <c r="V3" s="6" t="inlineStr">
         <is>
           <t>2026-10-19T06:00:00Z</t>
         </is>
       </c>
-      <c r="W11" s="3" t="inlineStr">
+      <c r="W3" s="6" t="inlineStr">
         <is>
           <t>19-10-2026 11:30:00</t>
         </is>
       </c>
-      <c r="X11" s="3" t="inlineStr">
+      <c r="X3" s="4" t="inlineStr">
         <is>
           <t>hi</t>
         </is>
       </c>
-      <c r="Y11" s="3" t="inlineStr">
+      <c r="Y3" s="4" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="Z11" s="3" t="inlineStr">
+      <c r="Z3" s="6" t="inlineStr">
         <is>
           <t>Concerned team @MVVNLHQ, कृपया सम्मानित उपभोक्ता की बिजली आपूर्ति बाधित होने की शिकायत का संज्ञान लेकर आवश्यक कार्यवाही करें।</t>
         </is>
       </c>
-      <c r="AA11" s="3" t="inlineStr">
+      <c r="AA3" s="4" t="inlineStr">
         <is>
           <t>DRAFT_READY</t>
         </is>
       </c>
-      <c r="AB11" s="3" t="inlineStr"/>
-      <c r="AC11" s="3" t="inlineStr"/>
-      <c r="AD11" s="3" t="inlineStr"/>
-      <c r="AE11" s="3" t="inlineStr">
+      <c r="AB3" s="6" t="inlineStr"/>
+      <c r="AC3" s="6" t="inlineStr"/>
+      <c r="AD3" s="6" t="inlineStr"/>
+      <c r="AE3" s="4" t="inlineStr">
         <is>
           <t>CLASSIFIED</t>
         </is>
       </c>
-      <c r="AF11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="AF3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4" ht="45" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>19-10-2026</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>MORNING</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>MORNING</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>https://x.com/drx_mohd_sami/status/2111617408557568279?s=20</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>drx_mohd_sami</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>upl</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr"/>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>SUPPLY_OUTAGE</t>
         </is>
       </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>PVVNL</t>
         </is>
       </c>
-      <c r="L12" s="3" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>BULANDSAHAR</t>
         </is>
       </c>
-      <c r="M12" s="3" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>BULANDSAHAR</t>
         </is>
       </c>
-      <c r="N12" s="3" t="inlineStr">
+      <c r="N4" s="6" t="inlineStr">
         <is>
           <t>Verified match for BULANDSAHAR -&gt; PVVNL</t>
         </is>
       </c>
-      <c r="O12" s="3" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>Forwarded to Discom</t>
         </is>
       </c>
-      <c r="P12" s="3" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="Q12" s="3" t="inlineStr"/>
-      <c r="R12" s="3" t="inlineStr"/>
-      <c r="S12" s="3" t="inlineStr"/>
-      <c r="T12" s="3" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr"/>
+      <c r="R4" s="4" t="inlineStr"/>
+      <c r="S4" s="4" t="inlineStr"/>
+      <c r="T4" s="6" t="inlineStr">
         <is>
           <t>2111617408557568279</t>
         </is>
       </c>
-      <c r="U12" s="3" t="inlineStr">
+      <c r="U4" s="6" t="inlineStr">
         <is>
           <t>@UPPCLLKO @PVVNLHQ Bulandshahr city power outage since 2 PM. Inverter batteries dying, please restore supply immediately.</t>
         </is>
       </c>
-      <c r="V12" s="3" t="inlineStr">
+      <c r="V4" s="6" t="inlineStr">
         <is>
           <t>2026-10-19T06:15:00Z</t>
         </is>
       </c>
-      <c r="W12" s="3" t="inlineStr">
+      <c r="W4" s="6" t="inlineStr">
         <is>
           <t>19-10-2026 11:45:00</t>
         </is>
       </c>
-      <c r="X12" s="3" t="inlineStr">
+      <c r="X4" s="4" t="inlineStr">
         <is>
           <t>en</t>
         </is>
       </c>
-      <c r="Y12" s="3" t="inlineStr">
+      <c r="Y4" s="4" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="Z12" s="3" t="inlineStr">
+      <c r="Z4" s="6" t="inlineStr">
         <is>
           <t>Concerned team @PVVNLHQ, kindly look into this consumer power supply outage grievance and take prompt action.</t>
         </is>
       </c>
-      <c r="AA12" s="3" t="inlineStr">
+      <c r="AA4" s="4" t="inlineStr">
         <is>
           <t>DRAFT_READY</t>
         </is>
       </c>
-      <c r="AB12" s="3" t="inlineStr"/>
-      <c r="AC12" s="3" t="inlineStr"/>
-      <c r="AD12" s="3" t="inlineStr"/>
-      <c r="AE12" s="3" t="inlineStr">
+      <c r="AB4" s="6" t="inlineStr"/>
+      <c r="AC4" s="6" t="inlineStr"/>
+      <c r="AD4" s="6" t="inlineStr"/>
+      <c r="AE4" s="4" t="inlineStr">
         <is>
           <t>CLASSIFIED</t>
         </is>
       </c>
-      <c r="AF12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="AF4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5" ht="45" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>19-10-2026</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>MORNING</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>MORNING</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>https://x.com/durgeshkumabq8/status/2111609477049012326?s=20</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>durgeshkumabq8</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>akb</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr"/>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>TRANSFORMER_DAMAGE</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>MVVNL</t>
         </is>
       </c>
-      <c r="L13" s="3" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>AYODHYA</t>
         </is>
       </c>
-      <c r="M13" s="3" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>AYODHYA</t>
         </is>
       </c>
-      <c r="N13" s="3" t="inlineStr">
+      <c r="N5" s="6" t="inlineStr">
         <is>
           <t>Verified match for AYODHYA -&gt; MVVNL</t>
         </is>
       </c>
-      <c r="O13" s="3" t="inlineStr">
+      <c r="O5" s="4" t="inlineStr">
         <is>
           <t>Forwarded to Discom</t>
         </is>
       </c>
-      <c r="P13" s="3" t="inlineStr">
+      <c r="P5" s="4" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="Q13" s="3" t="inlineStr"/>
-      <c r="R13" s="3" t="inlineStr"/>
-      <c r="S13" s="3" t="inlineStr"/>
-      <c r="T13" s="3" t="inlineStr">
+      <c r="Q5" s="4" t="inlineStr"/>
+      <c r="R5" s="4" t="inlineStr"/>
+      <c r="S5" s="4" t="inlineStr"/>
+      <c r="T5" s="6" t="inlineStr">
         <is>
           <t>2111609477049012326</t>
         </is>
       </c>
-      <c r="U13" s="3" t="inlineStr">
+      <c r="U5" s="6" t="inlineStr">
         <is>
           <t>@aksharmaBharat @UPPCLLKO हमारे गांव में 63 KVA का ट्रांसफार्मर फुंक गया है। 3 दिन से अंधेरा है। नया ट्रांसफार्मर लगवाया जाए।</t>
         </is>
       </c>
-      <c r="V13" s="3" t="inlineStr">
+      <c r="V5" s="6" t="inlineStr">
         <is>
           <t>2026-10-19T06:20:00Z</t>
         </is>
       </c>
-      <c r="W13" s="3" t="inlineStr">
+      <c r="W5" s="6" t="inlineStr">
         <is>
           <t>19-10-2026 11:50:00</t>
         </is>
       </c>
-      <c r="X13" s="3" t="inlineStr">
+      <c r="X5" s="4" t="inlineStr">
         <is>
           <t>hi</t>
         </is>
       </c>
-      <c r="Y13" s="3" t="inlineStr">
+      <c r="Y5" s="4" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="Z13" s="3" t="inlineStr">
+      <c r="Z5" s="6" t="inlineStr">
         <is>
           <t>Concerned team @MVVNLHQ, कृपया क्षतिग्रस्त परिवर्तक (ट्रांसफार्मर) का अविलंब संज्ञान लेकर नियमानुसार आवश्यक कार्यवाही सुनिश्चित करें।</t>
         </is>
       </c>
-      <c r="AA13" s="3" t="inlineStr">
+      <c r="AA5" s="4" t="inlineStr">
         <is>
           <t>DRAFT_READY</t>
         </is>
       </c>
-      <c r="AB13" s="3" t="inlineStr"/>
-      <c r="AC13" s="3" t="inlineStr"/>
-      <c r="AD13" s="3" t="inlineStr"/>
-      <c r="AE13" s="3" t="inlineStr">
+      <c r="AB5" s="6" t="inlineStr"/>
+      <c r="AC5" s="6" t="inlineStr"/>
+      <c r="AD5" s="6" t="inlineStr"/>
+      <c r="AE5" s="4" t="inlineStr">
         <is>
           <t>CLASSIFIED</t>
         </is>
       </c>
-      <c r="AF13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="AF5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>19-10-2026</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>MORNING</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>MORNING</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>https://x.com/Er_Naushad_khan/status/2111626795447706058?s=20</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>Er_Naushad_khan</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>upl</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr"/>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr"/>
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>SUPPLY_VOLTAGE</t>
         </is>
       </c>
-      <c r="K14" s="3" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>KESCO</t>
         </is>
       </c>
-      <c r="L14" s="3" t="inlineStr">
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>KESCO</t>
         </is>
       </c>
-      <c r="M14" s="3" t="inlineStr">
+      <c r="M6" s="4" t="inlineStr">
         <is>
           <t>KANPUR CITY</t>
         </is>
       </c>
-      <c r="N14" s="3" t="inlineStr">
+      <c r="N6" s="6" t="inlineStr">
         <is>
           <t>Verified match for KANPUR CITY -&gt; KESCO</t>
         </is>
       </c>
-      <c r="O14" s="3" t="inlineStr">
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>Forwarded to Discom</t>
         </is>
       </c>
-      <c r="P14" s="3" t="inlineStr">
+      <c r="P6" s="4" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="Q14" s="3" t="inlineStr"/>
-      <c r="R14" s="3" t="inlineStr"/>
-      <c r="S14" s="3" t="inlineStr"/>
-      <c r="T14" s="3" t="inlineStr">
+      <c r="Q6" s="4" t="inlineStr"/>
+      <c r="R6" s="4" t="inlineStr"/>
+      <c r="S6" s="4" t="inlineStr"/>
+      <c r="T6" s="6" t="inlineStr">
         <is>
           <t>2111626795447706058</t>
         </is>
       </c>
-      <c r="U14" s="3" t="inlineStr">
+      <c r="U6" s="6" t="inlineStr">
         <is>
           <t>@UPPCLLKO @KESCoHQ Rawatpur Kanpur me heavy voltage fluctuation chal raha hai. Fridge and AC damaged. Please fix transformer.</t>
         </is>
       </c>
-      <c r="V14" s="3" t="inlineStr">
+      <c r="V6" s="6" t="inlineStr">
         <is>
           <t>2026-10-19T06:30:00Z</t>
         </is>
       </c>
-      <c r="W14" s="3" t="inlineStr">
+      <c r="W6" s="6" t="inlineStr">
         <is>
           <t>19-10-2026 12:00:00</t>
         </is>
       </c>
-      <c r="X14" s="3" t="inlineStr">
+      <c r="X6" s="4" t="inlineStr">
         <is>
           <t>hi-Latn</t>
         </is>
       </c>
-      <c r="Y14" s="3" t="inlineStr">
+      <c r="Y6" s="4" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="Z14" s="3" t="inlineStr">
+      <c r="Z6" s="6" t="inlineStr">
         <is>
           <t>Concerned team @KESCoHQ, कृपया वोल्टेज समस्या (लो/हाई वोल्टेज) का संज्ञान लेकर आपूर्ति को सामान्य कराना सुनिश्चित करें।</t>
         </is>
       </c>
-      <c r="AA14" s="3" t="inlineStr">
+      <c r="AA6" s="4" t="inlineStr">
         <is>
           <t>DRAFT_READY</t>
         </is>
       </c>
-      <c r="AB14" s="3" t="inlineStr"/>
-      <c r="AC14" s="3" t="inlineStr"/>
-      <c r="AD14" s="3" t="inlineStr"/>
-      <c r="AE14" s="3" t="inlineStr">
+      <c r="AB6" s="6" t="inlineStr"/>
+      <c r="AC6" s="6" t="inlineStr"/>
+      <c r="AD6" s="6" t="inlineStr"/>
+      <c r="AE6" s="4" t="inlineStr">
         <is>
           <t>CLASSIFIED</t>
         </is>
       </c>
-      <c r="AF14" s="3" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="AF6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>19-10-2026</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>MORNING</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>MORNING</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>https://x.com/rohi_tkushwahaa/status/2111631974771360067?s=20</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>rohi_tkushwahaa</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>upm</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr"/>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="J15" s="3" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>CONNECTION_NEW</t>
         </is>
       </c>
-      <c r="K15" s="3" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>PuVVNL</t>
         </is>
       </c>
-      <c r="L15" s="3" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>GORAKHPUR-2</t>
         </is>
       </c>
-      <c r="M15" s="3" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>DEORIA</t>
         </is>
       </c>
-      <c r="N15" s="3" t="inlineStr">
+      <c r="N7" s="6" t="inlineStr">
         <is>
           <t>Verified match for DEORIA -&gt; PuVVNL</t>
         </is>
       </c>
-      <c r="O15" s="3" t="inlineStr">
+      <c r="O7" s="4" t="inlineStr">
         <is>
           <t>Forwarded to Discom</t>
         </is>
       </c>
-      <c r="P15" s="3" t="inlineStr">
+      <c r="P7" s="4" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="Q15" s="3" t="inlineStr"/>
-      <c r="R15" s="3" t="inlineStr"/>
-      <c r="S15" s="3" t="inlineStr"/>
-      <c r="T15" s="3" t="inlineStr">
+      <c r="Q7" s="4" t="inlineStr"/>
+      <c r="R7" s="4" t="inlineStr"/>
+      <c r="S7" s="4" t="inlineStr"/>
+      <c r="T7" s="6" t="inlineStr">
         <is>
           <t>2111631974771360067</t>
         </is>
       </c>
-      <c r="U15" s="3" t="inlineStr">
+      <c r="U7" s="6" t="inlineStr">
         <is>
           <t>@mduppcl @PuVVNLHQ देवरिया में झटपट पोर्टल पर नए कनेक्शन के लिए 15 दिन पहले अप्लाई किया था लेकिन अभी तक मीटर नहीं लगा।</t>
         </is>
       </c>
-      <c r="V15" s="3" t="inlineStr">
+      <c r="V7" s="6" t="inlineStr">
         <is>
           <t>2026-10-19T06:40:00Z</t>
         </is>
       </c>
-      <c r="W15" s="3" t="inlineStr">
+      <c r="W7" s="6" t="inlineStr">
         <is>
           <t>19-10-2026 12:10:00</t>
         </is>
       </c>
-      <c r="X15" s="3" t="inlineStr">
+      <c r="X7" s="4" t="inlineStr">
         <is>
           <t>hi</t>
         </is>
       </c>
-      <c r="Y15" s="3" t="inlineStr">
+      <c r="Y7" s="4" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="Z15" s="3" t="inlineStr">
+      <c r="Z7" s="6" t="inlineStr">
         <is>
           <t>Concerned team @PuVVNLHQ, कृपया नवीन संयोजन (नए कनेक्शन) सम्बन्धी इस प्रकरण का संज्ञान लेकर आवश्यक कार्यवाही करें।</t>
         </is>
       </c>
-      <c r="AA15" s="3" t="inlineStr">
+      <c r="AA7" s="4" t="inlineStr">
         <is>
           <t>DRAFT_READY</t>
         </is>
       </c>
-      <c r="AB15" s="3" t="inlineStr"/>
-      <c r="AC15" s="3" t="inlineStr"/>
-      <c r="AD15" s="3" t="inlineStr"/>
-      <c r="AE15" s="3" t="inlineStr">
+      <c r="AB7" s="6" t="inlineStr"/>
+      <c r="AC7" s="6" t="inlineStr"/>
+      <c r="AD7" s="6" t="inlineStr"/>
+      <c r="AE7" s="4" t="inlineStr">
         <is>
           <t>CLASSIFIED</t>
         </is>
       </c>
-      <c r="AF15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="AF7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>19-10-2026</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>MORNING</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>MORNING</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>https://x.com/PooranSardar/status/2111658518130642993?s=20</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>PooranSardar</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>upl</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr"/>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr"/>
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr">
+      <c r="J8" s="4" t="inlineStr">
         <is>
           <t>BILL_RELATED</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>DVVNL</t>
         </is>
       </c>
-      <c r="L16" s="3" t="inlineStr">
+      <c r="L8" s="4" t="inlineStr">
         <is>
           <t>MATHURA</t>
         </is>
       </c>
-      <c r="M16" s="3" t="inlineStr">
+      <c r="M8" s="4" t="inlineStr">
         <is>
           <t>MATHURA</t>
         </is>
       </c>
-      <c r="N16" s="3" t="inlineStr">
+      <c r="N8" s="6" t="inlineStr">
         <is>
           <t>Verified match for MATHURA -&gt; DVVNL</t>
         </is>
       </c>
-      <c r="O16" s="3" t="inlineStr">
+      <c r="O8" s="4" t="inlineStr">
         <is>
           <t>Forwarded to Discom</t>
         </is>
       </c>
-      <c r="P16" s="3" t="inlineStr">
+      <c r="P8" s="4" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="Q16" s="3" t="inlineStr"/>
-      <c r="R16" s="3" t="inlineStr"/>
-      <c r="S16" s="3" t="inlineStr"/>
-      <c r="T16" s="3" t="inlineStr">
+      <c r="Q8" s="4" t="inlineStr"/>
+      <c r="R8" s="4" t="inlineStr"/>
+      <c r="S8" s="4" t="inlineStr"/>
+      <c r="T8" s="6" t="inlineStr">
         <is>
           <t>2111658518130642993</t>
         </is>
       </c>
-      <c r="U16" s="3" t="inlineStr">
+      <c r="U8" s="6" t="inlineStr">
         <is>
           <t>@UPPCLLKO @dvvnlhq मथुरा छाता क्षेत्र में अत्यधिक गलत बिल भेज दिया गया है। 2 कमरे के घर का बिल 45000 आया है।</t>
         </is>
       </c>
-      <c r="V16" s="3" t="inlineStr">
+      <c r="V8" s="6" t="inlineStr">
         <is>
           <t>2026-10-19T06:45:00Z</t>
         </is>
       </c>
-      <c r="W16" s="3" t="inlineStr">
+      <c r="W8" s="6" t="inlineStr">
         <is>
           <t>19-10-2026 12:15:00</t>
         </is>
       </c>
-      <c r="X16" s="3" t="inlineStr">
+      <c r="X8" s="4" t="inlineStr">
         <is>
           <t>hi</t>
         </is>
       </c>
-      <c r="Y16" s="3" t="inlineStr">
+      <c r="Y8" s="4" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="Z16" s="3" t="inlineStr">
+      <c r="Z8" s="6" t="inlineStr">
         <is>
           <t>Concerned team @dvvnlhq, कृपया सम्मानित उपभोक्ता की बिल सम्बन्धी शिकायत का संज्ञान लेकर त्वरित निस्तारण सुनिश्चित करें।</t>
         </is>
       </c>
-      <c r="AA16" s="3" t="inlineStr">
+      <c r="AA8" s="4" t="inlineStr">
         <is>
           <t>DRAFT_READY</t>
         </is>
       </c>
-      <c r="AB16" s="3" t="inlineStr"/>
-      <c r="AC16" s="3" t="inlineStr"/>
-      <c r="AD16" s="3" t="inlineStr"/>
-      <c r="AE16" s="3" t="inlineStr">
+      <c r="AB8" s="6" t="inlineStr"/>
+      <c r="AC8" s="6" t="inlineStr"/>
+      <c r="AD8" s="6" t="inlineStr"/>
+      <c r="AE8" s="4" t="inlineStr">
         <is>
           <t>CLASSIFIED</t>
         </is>
       </c>
-      <c r="AF16" s="3" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="AF8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>19-10-2026</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>MORNING</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>MORNING</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>https://x.com/Neeraj120459/status/2111660825899323771?s=20</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>Neeraj120459</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>upm</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr"/>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>APPRECIATION</t>
         </is>
       </c>
-      <c r="J17" s="3" t="inlineStr"/>
-      <c r="K17" s="3" t="inlineStr"/>
-      <c r="L17" s="3" t="inlineStr"/>
-      <c r="M17" s="3" t="inlineStr"/>
-      <c r="N17" s="3" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr"/>
+      <c r="K9" s="4" t="inlineStr"/>
+      <c r="L9" s="4" t="inlineStr"/>
+      <c r="M9" s="4" t="inlineStr"/>
+      <c r="N9" s="6" t="inlineStr">
         <is>
           <t>Consumer appreciation logged</t>
         </is>
       </c>
-      <c r="O17" s="3" t="inlineStr"/>
-      <c r="P17" s="3" t="inlineStr"/>
-      <c r="Q17" s="3" t="inlineStr"/>
-      <c r="R17" s="3" t="inlineStr"/>
-      <c r="S17" s="3" t="inlineStr"/>
-      <c r="T17" s="3" t="inlineStr">
+      <c r="O9" s="4" t="inlineStr"/>
+      <c r="P9" s="4" t="inlineStr"/>
+      <c r="Q9" s="4" t="inlineStr"/>
+      <c r="R9" s="4" t="inlineStr"/>
+      <c r="S9" s="4" t="inlineStr"/>
+      <c r="T9" s="6" t="inlineStr">
         <is>
           <t>2111660825899323771</t>
         </is>
       </c>
-      <c r="U17" s="3" t="inlineStr">
+      <c r="U9" s="6" t="inlineStr">
         <is>
           <t>@UPPCLLKO @mduppcl Gomti Nagar sub station team resolved my fuse blown complaint within 30 minutes! Excellent work and thank you!</t>
         </is>
       </c>
-      <c r="V17" s="3" t="inlineStr">
+      <c r="V9" s="6" t="inlineStr">
         <is>
           <t>2026-10-19T06:50:00Z</t>
         </is>
       </c>
-      <c r="W17" s="3" t="inlineStr">
+      <c r="W9" s="6" t="inlineStr">
         <is>
           <t>19-10-2026 12:20:00</t>
         </is>
       </c>
-      <c r="X17" s="3" t="inlineStr">
+      <c r="X9" s="4" t="inlineStr">
         <is>
           <t>en</t>
         </is>
       </c>
-      <c r="Y17" s="3" t="inlineStr">
+      <c r="Y9" s="4" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="Z17" s="3" t="inlineStr"/>
-      <c r="AA17" s="3" t="inlineStr">
+      <c r="Z9" s="6" t="inlineStr"/>
+      <c r="AA9" s="4" t="inlineStr">
         <is>
           <t>SKIPPED</t>
         </is>
       </c>
-      <c r="AB17" s="3" t="inlineStr"/>
-      <c r="AC17" s="3" t="inlineStr"/>
-      <c r="AD17" s="3" t="inlineStr"/>
-      <c r="AE17" s="3" t="inlineStr">
+      <c r="AB9" s="6" t="inlineStr"/>
+      <c r="AC9" s="6" t="inlineStr"/>
+      <c r="AD9" s="6" t="inlineStr"/>
+      <c r="AE9" s="4" t="inlineStr">
         <is>
           <t>CLASSIFIED</t>
         </is>
       </c>
-      <c r="AF17" s="3" t="inlineStr"/>
+      <c r="AF9" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1589,1298 +1630,1298 @@
   <dimension ref="A1:C76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>DISCOM</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>District</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>ZONE</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>DVVNL</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>AGRA</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>AGRA-1</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>DVVNL</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>ALIGARH</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>ALIGARH</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>DVVNL</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>AURAIYA</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>KANPUR-2</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>DVVNL</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>BANDA</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>BANDA</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>DVVNL</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>CHITRAKOOT</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>BANDA</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>DVVNL</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>ETAH</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>ETAH</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>DVVNL</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>ETAWAH</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>KANPUR-2</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>DVVNL</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>FARRUKHABAD</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>KANPUR-2</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>DVVNL</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>FIROZABAD</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>FIROZABAD</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>DVVNL</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>HAMIRPUR</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>BANDA</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>DVVNL</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>HATHRAS</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>ETAH</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>DVVNL</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>JALAUN</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>JHANSI</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>DVVNL</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>JHANSI</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>JHANSI</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>DVVNL</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>KANNAUJ</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>KANPUR-2</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>DVVNL</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>KANPUR DEHAT</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>KANPUR-1</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>DVVNL</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>KASGANJ</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>ETAH</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>DVVNL</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>LALITPUR</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>JHANSI</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>DVVNL</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>MAHOBA</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>BANDA</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>DVVNL</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>MAINPURI</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>FIROZABAD</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>DVVNL</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>MATHURA</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>MATHURA</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>KESCO</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>KANPUR CITY</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>KESCO</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>MVVNL</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>AMBEDKAR NAGAR</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>AYODHYA</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>MVVNL</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>AMETHI</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>AYODHYA</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>MVVNL</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>AYODHYA</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>AYODHYA</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>MVVNL</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>BADAUN</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>BAREILY-2</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>MVVNL</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>BAHRAICH</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>DEVIPATAN</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="7" t="inlineStr">
         <is>
           <t>MVVNL</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>BALRAMPUR</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="7" t="inlineStr">
         <is>
           <t>DEVIPATAN</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="7" t="inlineStr">
         <is>
           <t>MVVNL</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>BARABANKI</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>AYODHYA</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="7" t="inlineStr">
         <is>
           <t>MVVNL</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="7" t="inlineStr">
         <is>
           <t>BAREILY</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="7" t="inlineStr">
         <is>
           <t>BAREILY-1</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>MVVNL</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>GONDA</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>DEVIPATAN</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>MVVNL</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="7" t="inlineStr">
         <is>
           <t>HARDOI</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="7" t="inlineStr">
         <is>
           <t>SITAPUR</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>MVVNL</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>LAKHIMPUR</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>SITAPUR</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="7" t="inlineStr">
         <is>
           <t>MVVNL</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="7" t="inlineStr">
         <is>
           <t>LUCKNOW</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="7" t="inlineStr">
         <is>
           <t>LESA</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="7" t="inlineStr">
         <is>
           <t>MVVNL</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="7" t="inlineStr">
         <is>
           <t>PILIBHIT</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="7" t="inlineStr">
         <is>
           <t>BAREILY-2</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="7" t="inlineStr">
         <is>
           <t>MVVNL</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="7" t="inlineStr">
         <is>
           <t>RAEBAREILY</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="7" t="inlineStr">
         <is>
           <t>RAEBAREILY</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="7" t="inlineStr">
         <is>
           <t>MVVNL</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>SHAJAHANPUR</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>BAREILY-2</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="7" t="inlineStr">
         <is>
           <t>MVVNL</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="7" t="inlineStr">
         <is>
           <t>SHRAVASTI</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="7" t="inlineStr">
         <is>
           <t>DEVIPATAN</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="7" t="inlineStr">
         <is>
           <t>MVVNL</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="7" t="inlineStr">
         <is>
           <t>SITAPUR</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="7" t="inlineStr">
         <is>
           <t>SITAPUR</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="7" t="inlineStr">
         <is>
           <t>MVVNL</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="7" t="inlineStr">
         <is>
           <t>SULTANPUR</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="7" t="inlineStr">
         <is>
           <t>AYODHYA</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="7" t="inlineStr">
         <is>
           <t>MVVNL</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="7" t="inlineStr">
         <is>
           <t>UNNAO</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="7" t="inlineStr">
         <is>
           <t>RAEBAREILY</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="7" t="inlineStr">
         <is>
           <t>PVVNL</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="7" t="inlineStr">
         <is>
           <t>AMROHA</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="7" t="inlineStr">
         <is>
           <t>GAZRAULA</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="7" t="inlineStr">
         <is>
           <t>PVVNL</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="7" t="inlineStr">
         <is>
           <t>BAGHPAT</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="7" t="inlineStr">
         <is>
           <t>MEERUT-2</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="7" t="inlineStr">
         <is>
           <t>PVVNL</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="7" t="inlineStr">
         <is>
           <t>BIJNOR</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="7" t="inlineStr">
         <is>
           <t>GAZRAULA</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="7" t="inlineStr">
         <is>
           <t>PVVNL</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="7" t="inlineStr">
         <is>
           <t>BULANDSAHAR</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="7" t="inlineStr">
         <is>
           <t>BULANDSAHAR</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="7" t="inlineStr">
         <is>
           <t>PVVNL</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="7" t="inlineStr">
         <is>
           <t>GAUTAM BUDH NAGAR</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="7" t="inlineStr">
         <is>
           <t>NOIDA</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="7" t="inlineStr">
         <is>
           <t>PVVNL</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="7" t="inlineStr">
         <is>
           <t>GHAZIABAD</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="7" t="inlineStr">
         <is>
           <t>GHAZIABAD</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="7" t="inlineStr">
         <is>
           <t>PVVNL</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="7" t="inlineStr">
         <is>
           <t>HAPUR</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="7" t="inlineStr">
         <is>
           <t>BULANDSAHAR</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="7" t="inlineStr">
         <is>
           <t>PVVNL</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="7" t="inlineStr">
         <is>
           <t>MEERUT</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="7" t="inlineStr">
         <is>
           <t>MEERUT</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="7" t="inlineStr">
         <is>
           <t>PVVNL</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B50" s="7" t="inlineStr">
         <is>
           <t>MORADABAD</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="7" t="inlineStr">
         <is>
           <t>MORADABAD</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="7" t="inlineStr">
         <is>
           <t>PVVNL</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="7" t="inlineStr">
         <is>
           <t>MUZAFFERNAGAR</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="7" t="inlineStr">
         <is>
           <t>MUZAFFERNAGAR</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="7" t="inlineStr">
         <is>
           <t>PVVNL</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B52" s="7" t="inlineStr">
         <is>
           <t>RAMPUR</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="7" t="inlineStr">
         <is>
           <t>MORADABAD</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="7" t="inlineStr">
         <is>
           <t>PVVNL</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B53" s="7" t="inlineStr">
         <is>
           <t>SAHARANPUR</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="7" t="inlineStr">
         <is>
           <t>SAHARANPUR</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="7" t="inlineStr">
         <is>
           <t>PVVNL</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="7" t="inlineStr">
         <is>
           <t>SAMBHAL</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="7" t="inlineStr">
         <is>
           <t>MORADABAD</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="7" t="inlineStr">
         <is>
           <t>PVVNL</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B55" s="7" t="inlineStr">
         <is>
           <t>SHAMLI</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="7" t="inlineStr">
         <is>
           <t>MUZAFFERNAGAR</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="7" t="inlineStr">
         <is>
           <t>PuVVNL</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B56" s="7" t="inlineStr">
         <is>
           <t>AZAMGARH</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C56" s="7" t="inlineStr">
         <is>
           <t>AZAMGARH</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="7" t="inlineStr">
         <is>
           <t>PuVVNL</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B57" s="7" t="inlineStr">
         <is>
           <t>BALLIA</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C57" s="7" t="inlineStr">
         <is>
           <t>AZAMGARH</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="7" t="inlineStr">
         <is>
           <t>PuVVNL</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B58" s="7" t="inlineStr">
         <is>
           <t>BASTI</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="7" t="inlineStr">
         <is>
           <t>BASTI</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="A59" s="7" t="inlineStr">
         <is>
           <t>PuVVNL</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B59" s="7" t="inlineStr">
         <is>
           <t>BHADOHI</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="7" t="inlineStr">
         <is>
           <t>MIRZAPUR</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="A60" s="7" t="inlineStr">
         <is>
           <t>PuVVNL</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B60" s="7" t="inlineStr">
         <is>
           <t>CHANDAULI</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C60" s="7" t="inlineStr">
         <is>
           <t>VARANASI-2</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" s="7" t="inlineStr">
         <is>
           <t>PuVVNL</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B61" s="7" t="inlineStr">
         <is>
           <t>DEORIA</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="7" t="inlineStr">
         <is>
           <t>GORAKHPUR-2</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="7" t="inlineStr">
         <is>
           <t>PuVVNL</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B62" s="7" t="inlineStr">
         <is>
           <t>FATEHPUR</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C62" s="7" t="inlineStr">
         <is>
           <t>PRAYAGRAJ-2</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="7" t="inlineStr">
         <is>
           <t>PuVVNL</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B63" s="7" t="inlineStr">
         <is>
           <t>GHAZIPUR</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C63" s="7" t="inlineStr">
         <is>
           <t>VARANASI-2</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="7" t="inlineStr">
         <is>
           <t>PuVVNL</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B64" s="7" t="inlineStr">
         <is>
           <t>GORAKHPUR</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="7" t="inlineStr">
         <is>
           <t>GORAKHPUR-1</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" s="7" t="inlineStr">
         <is>
           <t>PuVVNL</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B65" s="7" t="inlineStr">
         <is>
           <t>JAUNPUR</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C65" s="7" t="inlineStr">
         <is>
           <t>VARANASI-2</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" s="7" t="inlineStr">
         <is>
           <t>PuVVNL</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B66" s="7" t="inlineStr">
         <is>
           <t>KAUSHAMBI</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C66" s="7" t="inlineStr">
         <is>
           <t>PRAYAGRAJ-2</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
+      <c r="A67" s="7" t="inlineStr">
         <is>
           <t>PuVVNL</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
+      <c r="B67" s="7" t="inlineStr">
         <is>
           <t>KUSHINAGAR</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C67" s="7" t="inlineStr">
         <is>
           <t>GORAKHPUR-2</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
+      <c r="A68" s="7" t="inlineStr">
         <is>
           <t>PuVVNL</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B68" s="7" t="inlineStr">
         <is>
           <t>MAHARAJGANJ</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C68" s="7" t="inlineStr">
         <is>
           <t>GORAKHPUR-2</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="7" t="inlineStr">
         <is>
           <t>PuVVNL</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B69" s="7" t="inlineStr">
         <is>
           <t>MAU</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C69" s="7" t="inlineStr">
         <is>
           <t>AZAMGARH</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
+      <c r="A70" s="7" t="inlineStr">
         <is>
           <t>PuVVNL</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
+      <c r="B70" s="7" t="inlineStr">
         <is>
           <t>MIRZAPUR</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="C70" s="7" t="inlineStr">
         <is>
           <t>MIRZAPUR</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
+      <c r="A71" s="7" t="inlineStr">
         <is>
           <t>PuVVNL</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
+      <c r="B71" s="7" t="inlineStr">
         <is>
           <t>PRATAPGARH</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
+      <c r="C71" s="7" t="inlineStr">
         <is>
           <t>PRAYAGRAJ-2</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
+      <c r="A72" s="7" t="inlineStr">
         <is>
           <t>PuVVNL</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B72" s="7" t="inlineStr">
         <is>
           <t>PRAYAGRAJ</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C72" s="7" t="inlineStr">
         <is>
           <t>PRAYAGRAJ-1</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
+      <c r="A73" s="7" t="inlineStr">
         <is>
           <t>PuVVNL</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
+      <c r="B73" s="7" t="inlineStr">
         <is>
           <t>SANT KABIR NAGAR</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C73" s="7" t="inlineStr">
         <is>
           <t>BASTI</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
+      <c r="A74" s="7" t="inlineStr">
         <is>
           <t>PuVVNL</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
+      <c r="B74" s="7" t="inlineStr">
         <is>
           <t>SIDDHARTH NAGAR</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C74" s="7" t="inlineStr">
         <is>
           <t>BASTI</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
+      <c r="A75" s="7" t="inlineStr">
         <is>
           <t>PuVVNL</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B75" s="7" t="inlineStr">
         <is>
           <t>SONBHADRA</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C75" s="7" t="inlineStr">
         <is>
           <t>MIRZAPUR</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
+      <c r="A76" s="7" t="inlineStr">
         <is>
           <t>PuVVNL</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="B76" s="7" t="inlineStr">
         <is>
           <t>VARANASI</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C76" s="7" t="inlineStr">
         <is>
           <t>VARANASI-1</t>
         </is>
@@ -2900,125 +2941,125 @@
   <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>SETTING_KEY</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>VALUE</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>DESCRIPTION</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>EMERGENCY_STOP</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Global kill-switch. When TRUE, no polling or replies run.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>AUTO_POST_ENABLED</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>When FALSE, replies only draft and require manual approval.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>DAILY_POST_CAP</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>Maximum automated replies permitted per calendar day.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>POLLING_INTERVAL_MINS</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Frequency of background post monitoring cycles.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>ALLOWED_DISCOMS</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>@PVVNLHQ, @dvvnlhq, @PuVVNLHQ, @KESCoHQ, @MVVNLHQ</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>Safety allowlist of receiving handles.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>MONITORED_APEX</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>@UPPCLLKO, @EMofficeUP, @AKSharmaOffice, @aksharmaBharat, @ChairmanUppcl, @mduppcl</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Monitored accounts.</t>
         </is>
@@ -3038,206 +3079,206 @@
   <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="49" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>UPPCL X COMPLAINT MONITORING DASHBOARD (TRIAL)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="10" t="inlineStr">
         <is>
           <t>Source / Category</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Total Complaints Recorded</t>
         </is>
       </c>
-      <c r="B3">
-        <f>COUNTA('Twitter Complaint List'!E11:E50)</f>
+      <c r="B3" s="7">
+        <f>COUNTA('Twitter Complaint List'!E3:E100)</f>
         <v/>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Active post links count</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Supply Outages</t>
         </is>
       </c>
-      <c r="B4">
-        <f>COUNTIF('Twitter Complaint List'!J11:J50, "SUPPLY_OUTAGE")</f>
+      <c r="B4" s="7">
+        <f>COUNTIF('Twitter Complaint List'!J3:J100, "SUPPLY_OUTAGE")</f>
         <v/>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>SUPPLY_OUTAGE</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Transformer Damage</t>
         </is>
       </c>
-      <c r="B5">
-        <f>COUNTIF('Twitter Complaint List'!J11:J50, "TRANSFORMER_DAMAGE")</f>
+      <c r="B5" s="7">
+        <f>COUNTIF('Twitter Complaint List'!J3:J100, "TRANSFORMER_DAMAGE")</f>
         <v/>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>TRANSFORMER_DAMAGE</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Billing Issues</t>
         </is>
       </c>
-      <c r="B6">
-        <f>COUNTIF('Twitter Complaint List'!J11:J50, "BILL_RELATED")</f>
+      <c r="B6" s="7">
+        <f>COUNTIF('Twitter Complaint List'!J3:J100, "BILL_RELATED")</f>
         <v/>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>BILL_RELATED</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Voltage Fluctuations</t>
         </is>
       </c>
-      <c r="B7">
-        <f>COUNTIF('Twitter Complaint List'!J11:J50, "SUPPLY_VOLTAGE")</f>
+      <c r="B7" s="7">
+        <f>COUNTIF('Twitter Complaint List'!J3:J100, "SUPPLY_VOLTAGE")</f>
         <v/>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>SUPPLY_VOLTAGE</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>New Connection Issues</t>
         </is>
       </c>
-      <c r="B8">
-        <f>COUNTIF('Twitter Complaint List'!J11:J50, "CONNECTION_NEW")</f>
+      <c r="B8" s="7">
+        <f>COUNTIF('Twitter Complaint List'!J3:J100, "CONNECTION_NEW")</f>
         <v/>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>CONNECTION_NEW</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>MVVNL Complaints</t>
         </is>
       </c>
-      <c r="B9">
-        <f>COUNTIF('Twitter Complaint List'!K11:K50, "MVVNL")</f>
+      <c r="B9" s="7">
+        <f>COUNTIF('Twitter Complaint List'!K3:K100, "MVVNL")</f>
         <v/>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Central UP</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>PVVNL Complaints</t>
         </is>
       </c>
-      <c r="B10">
-        <f>COUNTIF('Twitter Complaint List'!K11:K50, "PVVNL")</f>
+      <c r="B10" s="7">
+        <f>COUNTIF('Twitter Complaint List'!K3:K100, "PVVNL")</f>
         <v/>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>Western UP</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>PuVVNL Complaints</t>
         </is>
       </c>
-      <c r="B11">
-        <f>COUNTIF('Twitter Complaint List'!K11:K50, "PuVVNL")</f>
+      <c r="B11" s="7">
+        <f>COUNTIF('Twitter Complaint List'!K3:K100, "PuVVNL")</f>
         <v/>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Eastern UP</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>DVVNL Complaints</t>
         </is>
       </c>
-      <c r="B12">
-        <f>COUNTIF('Twitter Complaint List'!K11:K50, "DVVNL")</f>
+      <c r="B12" s="7">
+        <f>COUNTIF('Twitter Complaint List'!K3:K100, "DVVNL")</f>
         <v/>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Southern UP</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>KESCo Complaints</t>
         </is>
       </c>
-      <c r="B13">
-        <f>COUNTIF('Twitter Complaint List'!K11:K50, "KESCO")</f>
+      <c r="B13" s="7">
+        <f>COUNTIF('Twitter Complaint List'!K3:K100, "KESCO")</f>
         <v/>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Kanpur City</t>
         </is>

</xml_diff>